<commit_message>
paper run 2026-08-29 13:27
</commit_message>
<xml_diff>
--- a/reports/2026-08-29.xlsx
+++ b/reports/2026-08-29.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,158 +628,253 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По активам</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>По часам</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>

<commit_message>
paper run 2026-08-29 19:07
</commit_message>
<xml_diff>
--- a/reports/2026-08-29.xlsx
+++ b/reports/2026-08-29.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,13 +632,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>7.85</v>
+        <v>6.6</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -658,13 +658,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>4.08</v>
+        <v>2.83</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -703,13 +703,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>7.85</v>
+        <v>3.24</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -718,163 +718,182 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>NO_LIQUIDITY</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>2</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>По часам</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>

<commit_message>
paper run 2026-08-30 00:48
</commit_message>
<xml_diff>
--- a/reports/2026-08-29.xlsx
+++ b/reports/2026-08-29.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -647,43 +647,43 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" t="n">
-        <v>2.83</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>3.77</v>
+        <v>6.59</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -692,43 +692,43 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>3</v>
-      </c>
-      <c r="C20" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>3.36</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -737,163 +737,182 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>NO_LIQUIDITY</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" t="n">
         <v>4</v>
       </c>
-      <c r="C23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D23" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="D24" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>По часам</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>